<commit_message>
add province patent count graph
</commit_message>
<xml_diff>
--- a/就业人口.xlsx
+++ b/就业人口.xlsx
@@ -1,25 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView windowWidth="29100" windowHeight="13540"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="43">
   <si>
-    <t>年度标识</t>
+    <t>年份</t>
   </si>
   <si>
-    <t>省份名称</t>
+    <t>省份</t>
   </si>
   <si>
     <t>就业人员</t>
@@ -148,33 +161,376 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -197,9 +553,251 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -207,11 +805,63 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -494,16 +1144,20 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:L769"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
+  <cols>
+    <col min="8" max="8" width="26.4423076923077" customWidth="1"/>
+    <col min="9" max="9" width="33.1730769230769" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="2:12">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -538,7 +1192,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:10">
       <c r="A2" s="1">
         <v>48</v>
       </c>
@@ -570,7 +1224,7 @@
         <v>27.5</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:10">
       <c r="A3" s="1">
         <v>49</v>
       </c>
@@ -602,7 +1256,7 @@
         <v>27.7</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:10">
       <c r="A4" s="1">
         <v>50</v>
       </c>
@@ -634,7 +1288,7 @@
         <v>28.6</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:10">
       <c r="A5" s="1">
         <v>51</v>
       </c>
@@ -666,7 +1320,7 @@
         <v>29.3</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:10">
       <c r="A6" s="1">
         <v>52</v>
       </c>
@@ -698,7 +1352,7 @@
         <v>30.6</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:10">
       <c r="A7" s="1">
         <v>53</v>
       </c>
@@ -730,7 +1384,7 @@
         <v>31.4</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:10">
       <c r="A8" s="1">
         <v>54</v>
       </c>
@@ -762,7 +1416,7 @@
         <v>32.2</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:10">
       <c r="A9" s="1">
         <v>55</v>
       </c>
@@ -794,7 +1448,7 @@
         <v>32.4</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:10">
       <c r="A10" s="1">
         <v>56</v>
       </c>
@@ -826,7 +1480,7 @@
         <v>33.2</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:10">
       <c r="A11" s="1">
         <v>57</v>
       </c>
@@ -858,7 +1512,7 @@
         <v>34.1</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:10">
       <c r="A12" s="1">
         <v>58</v>
       </c>
@@ -890,7 +1544,7 @@
         <v>34.6</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:10">
       <c r="A13" s="1">
         <v>59</v>
       </c>
@@ -922,7 +1576,7 @@
         <v>35.7</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:10">
       <c r="A14" s="1">
         <v>60</v>
       </c>
@@ -954,7 +1608,7 @@
         <v>36.1</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:10">
       <c r="A15" s="1">
         <v>61</v>
       </c>
@@ -986,7 +1640,7 @@
         <v>38.5</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:10">
       <c r="A16" s="1">
         <v>62</v>
       </c>
@@ -1320,7 +1974,7 @@
         <v>619.3</v>
       </c>
       <c r="E26">
-        <v>72.90000000000001</v>
+        <v>72.9</v>
       </c>
       <c r="F26">
         <v>208.2</v>
@@ -1384,7 +2038,7 @@
         <v>679.2</v>
       </c>
       <c r="E28">
-        <v>67.59999999999999</v>
+        <v>67.6</v>
       </c>
       <c r="F28">
         <v>235.3</v>
@@ -1495,7 +2149,7 @@
         <v>26.3</v>
       </c>
       <c r="J31">
-        <v>66.59999999999999</v>
+        <v>66.6</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -1527,7 +2181,7 @@
         <v>24.5</v>
       </c>
       <c r="J32">
-        <v>68.90000000000001</v>
+        <v>68.9</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -1591,7 +2245,7 @@
         <v>21.2</v>
       </c>
       <c r="J34">
-        <v>72.40000000000001</v>
+        <v>72.4</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -1655,7 +2309,7 @@
         <v>19.6</v>
       </c>
       <c r="J36">
-        <v>74.40000000000001</v>
+        <v>74.4</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -1719,7 +2373,7 @@
         <v>19.2</v>
       </c>
       <c r="J38">
-        <v>75.59999999999999</v>
+        <v>75.6</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -1847,7 +2501,7 @@
         <v>15.8</v>
       </c>
       <c r="J42">
-        <v>80.09999999999999</v>
+        <v>80.1</v>
       </c>
     </row>
     <row r="43" spans="1:10">
@@ -1879,7 +2533,7 @@
         <v>15.5</v>
       </c>
       <c r="J43">
-        <v>80.59999999999999</v>
+        <v>80.6</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -1911,7 +2565,7 @@
         <v>14.7</v>
       </c>
       <c r="J44">
-        <v>81.59999999999999</v>
+        <v>81.6</v>
       </c>
     </row>
     <row r="45" spans="1:10">
@@ -1943,7 +2597,7 @@
         <v>13.6</v>
       </c>
       <c r="J45">
-        <v>83.09999999999999</v>
+        <v>83.1</v>
       </c>
     </row>
     <row r="46" spans="1:10">
@@ -1975,7 +2629,7 @@
         <v>13.6</v>
       </c>
       <c r="J46">
-        <v>83.09999999999999</v>
+        <v>83.1</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -2088,7 +2742,7 @@
         <v>406.7</v>
       </c>
       <c r="E50">
-        <v>80.90000000000001</v>
+        <v>80.9</v>
       </c>
       <c r="F50">
         <v>166.8</v>
@@ -2248,7 +2902,7 @@
         <v>426.8802</v>
       </c>
       <c r="E55">
-        <v>80.52589999999999</v>
+        <v>80.5259</v>
       </c>
       <c r="F55">
         <v>173.2975</v>
@@ -2312,7 +2966,7 @@
         <v>432.736</v>
       </c>
       <c r="E57">
-        <v>77.85769999999999</v>
+        <v>77.8577</v>
       </c>
       <c r="F57">
         <v>181.2792</v>
@@ -2344,7 +2998,7 @@
         <v>503.1363</v>
       </c>
       <c r="E58">
-        <v>78.06999999999999</v>
+        <v>78.07</v>
       </c>
       <c r="F58">
         <v>203.9065</v>
@@ -2481,7 +3135,7 @@
         <v>346</v>
       </c>
       <c r="H62">
-        <v>8.802308802308801</v>
+        <v>8.8023088023088</v>
       </c>
       <c r="I62">
         <v>41.2698412698413</v>
@@ -2891,7 +3545,7 @@
         <v>1676.34</v>
       </c>
       <c r="F75">
-        <v>899.6799999999999</v>
+        <v>899.68</v>
       </c>
       <c r="G75">
         <v>833.14</v>
@@ -3022,7 +3676,7 @@
         <v>1043.56</v>
       </c>
       <c r="G79">
-        <v>960.6900000000001</v>
+        <v>960.69</v>
       </c>
       <c r="H79">
         <v>43.84</v>
@@ -3880,7 +4534,7 @@
         <v>1583.4558</v>
       </c>
       <c r="E106">
-        <v>642.8203999999999</v>
+        <v>642.8204</v>
       </c>
       <c r="F106">
         <v>417.3541</v>
@@ -4011,7 +4665,7 @@
         <v>608.79</v>
       </c>
       <c r="F110">
-        <v>517.1900000000001</v>
+        <v>517.19</v>
       </c>
       <c r="G110">
         <v>708.02</v>
@@ -4104,13 +4758,13 @@
         <v>1827</v>
       </c>
       <c r="E113">
-        <v>549.9299999999999</v>
+        <v>549.93</v>
       </c>
       <c r="F113">
         <v>467.89</v>
       </c>
       <c r="G113">
-        <v>809.1799999999999</v>
+        <v>809.18</v>
       </c>
       <c r="H113">
         <v>30.1002</v>
@@ -4206,7 +4860,7 @@
         <v>436.52</v>
       </c>
       <c r="G116">
-        <v>874.6900000000001</v>
+        <v>874.69</v>
       </c>
       <c r="H116">
         <v>26.7071</v>
@@ -5576,7 +6230,7 @@
         <v>2518.8756</v>
       </c>
       <c r="E159">
-        <v>683.8022999999999</v>
+        <v>683.8023</v>
       </c>
       <c r="F159">
         <v>724.1884</v>
@@ -6510,7 +7164,7 @@
         <v>205.24</v>
       </c>
       <c r="G188">
-        <v>600.1900000000001</v>
+        <v>600.19</v>
       </c>
       <c r="H188">
         <v>38.7044</v>
@@ -7496,7 +8150,7 @@
         <v>692.4</v>
       </c>
       <c r="E219">
-        <v>86.59999999999999</v>
+        <v>86.6</v>
       </c>
       <c r="F219">
         <v>288.7</v>
@@ -7601,7 +8255,7 @@
         <v>424.0036</v>
       </c>
       <c r="H222">
-        <v>8.288600000000001</v>
+        <v>8.2886</v>
       </c>
       <c r="I222">
         <v>39.5138</v>
@@ -7621,7 +8275,7 @@
         <v>20</v>
       </c>
       <c r="D223">
-        <v>855.8612000000001</v>
+        <v>855.8612</v>
       </c>
       <c r="E223">
         <v>61.0942</v>
@@ -8055,7 +8709,7 @@
         <v>30.7357922742538</v>
       </c>
       <c r="J236">
-        <v>66.29617783463939</v>
+        <v>66.2961778346394</v>
       </c>
     </row>
     <row r="237" spans="1:10">
@@ -8712,7 +9366,7 @@
         <v>4832.5</v>
       </c>
       <c r="E257">
-        <v>845.6900000000001</v>
+        <v>845.69</v>
       </c>
       <c r="F257">
         <v>2034.48</v>
@@ -8840,7 +9494,7 @@
         <v>4903.2</v>
       </c>
       <c r="E261">
-        <v>706.0599999999999</v>
+        <v>706.06</v>
       </c>
       <c r="F261">
         <v>1961.28</v>
@@ -9006,7 +9660,7 @@
         <v>966.3</v>
       </c>
       <c r="G266">
-        <v>789.8200000000001</v>
+        <v>789.82</v>
       </c>
       <c r="H266">
         <v>35.6</v>
@@ -9192,7 +9846,7 @@
         <v>3172.38</v>
       </c>
       <c r="E272">
-        <v>717.8099999999999</v>
+        <v>717.81</v>
       </c>
       <c r="F272">
         <v>1452.29</v>
@@ -9288,7 +9942,7 @@
         <v>3288.29</v>
       </c>
       <c r="E275">
-        <v>610.3200000000001</v>
+        <v>610.32</v>
       </c>
       <c r="F275">
         <v>1492.13</v>
@@ -9553,7 +10207,7 @@
         <v>1664.12</v>
       </c>
       <c r="H283">
-        <v>8.800000000000001</v>
+        <v>8.8</v>
       </c>
       <c r="I283">
         <v>45.1</v>
@@ -14027,7 +14681,7 @@
         <v>1458.5937</v>
       </c>
       <c r="F423">
-        <v>731.8784000000001</v>
+        <v>731.8784</v>
       </c>
       <c r="G423">
         <v>1213.5278</v>
@@ -14091,7 +14745,7 @@
         <v>1304.2078</v>
       </c>
       <c r="F425">
-        <v>774.7217000000001</v>
+        <v>774.7217</v>
       </c>
       <c r="G425">
         <v>1319.0705</v>
@@ -14219,7 +14873,7 @@
         <v>1107.2435</v>
       </c>
       <c r="F429">
-        <v>799.9930000000001</v>
+        <v>799.993</v>
       </c>
       <c r="G429">
         <v>1467.7635</v>
@@ -14475,7 +15129,7 @@
         <v>1961.93</v>
       </c>
       <c r="F437">
-        <v>790.6799999999999</v>
+        <v>790.68</v>
       </c>
       <c r="G437">
         <v>942.17</v>
@@ -14667,7 +15321,7 @@
         <v>1693.05</v>
       </c>
       <c r="F443">
-        <v>896.5700000000001</v>
+        <v>896.57</v>
       </c>
       <c r="G443">
         <v>1345.59</v>
@@ -14699,7 +15353,7 @@
         <v>1690.03</v>
       </c>
       <c r="F444">
-        <v>915.4299999999999</v>
+        <v>915.43</v>
       </c>
       <c r="G444">
         <v>1377.27</v>
@@ -14955,7 +15609,7 @@
         <v>1462.38</v>
       </c>
       <c r="F452">
-        <v>836.4400000000001</v>
+        <v>836.44</v>
       </c>
       <c r="G452">
         <v>1439.76</v>
@@ -15889,7 +16543,7 @@
         <v>3785</v>
       </c>
       <c r="H481">
-        <v>9.749185206178259</v>
+        <v>9.74918520617826</v>
       </c>
       <c r="I481">
         <v>36.6161258325067</v>
@@ -16241,7 +16895,7 @@
         <v>565</v>
       </c>
       <c r="H492">
-        <v>66.99169999999999</v>
+        <v>66.9917</v>
       </c>
       <c r="I492">
         <v>11.8155</v>
@@ -16692,7 +17346,7 @@
         <v>60.84</v>
       </c>
       <c r="I506">
-        <v>9.369999999999999</v>
+        <v>9.37</v>
       </c>
       <c r="J506">
         <v>29.79</v>
@@ -16724,7 +17378,7 @@
         <v>60.21</v>
       </c>
       <c r="I507">
-        <v>9.380000000000001</v>
+        <v>9.38</v>
       </c>
       <c r="J507">
         <v>30.42</v>
@@ -17163,7 +17817,7 @@
         <v>189.95</v>
       </c>
       <c r="F521">
-        <v>64.09999999999999</v>
+        <v>64.1</v>
       </c>
       <c r="G521">
         <v>256.71</v>
@@ -17608,7 +18262,7 @@
         <v>1456.3</v>
       </c>
       <c r="E535">
-        <v>678.3200000000001</v>
+        <v>678.32</v>
       </c>
       <c r="F535">
         <v>283.08</v>
@@ -17704,7 +18358,7 @@
         <v>1492.43</v>
       </c>
       <c r="E538">
-        <v>652.1900000000001</v>
+        <v>652.19</v>
       </c>
       <c r="F538">
         <v>307.66</v>
@@ -17774,7 +18428,7 @@
         <v>351.86</v>
       </c>
       <c r="G540">
-        <v>595.3200000000001</v>
+        <v>595.32</v>
       </c>
       <c r="H540">
         <v>38.9</v>
@@ -17832,7 +18486,7 @@
         <v>1605.89</v>
       </c>
       <c r="E542">
-        <v>531.1799999999999</v>
+        <v>531.18</v>
       </c>
       <c r="F542">
         <v>422.73</v>
@@ -18283,7 +18937,7 @@
         <v>2517.48</v>
       </c>
       <c r="F556">
-        <v>896.1799999999999</v>
+        <v>896.18</v>
       </c>
       <c r="G556">
         <v>1253.94</v>
@@ -19025,7 +19679,7 @@
         <v>241.8</v>
       </c>
       <c r="H579">
-        <v>81.83369999999999</v>
+        <v>81.8337</v>
       </c>
       <c r="I579">
         <v>6.4739</v>
@@ -19249,7 +19903,7 @@
         <v>336.15</v>
       </c>
       <c r="H586">
-        <v>72.31789999999999</v>
+        <v>72.3179</v>
       </c>
       <c r="I586">
         <v>9.6792</v>
@@ -19281,7 +19935,7 @@
         <v>345.03</v>
       </c>
       <c r="H587">
-        <v>70.54000000000001</v>
+        <v>70.54</v>
       </c>
       <c r="I587">
         <v>10.7279</v>
@@ -19793,10 +20447,10 @@
         <v>404.2</v>
       </c>
       <c r="H603">
-        <v>73.65000000000001</v>
+        <v>73.65</v>
       </c>
       <c r="I603">
-        <v>8.949999999999999</v>
+        <v>8.95</v>
       </c>
       <c r="J603">
         <v>17.4</v>
@@ -19825,7 +20479,7 @@
         <v>419</v>
       </c>
       <c r="H604">
-        <v>73.29000000000001</v>
+        <v>73.29</v>
       </c>
       <c r="I604">
         <v>8.82</v>
@@ -19889,7 +20543,7 @@
         <v>471.1</v>
       </c>
       <c r="H606">
-        <v>71.29000000000001</v>
+        <v>71.29</v>
       </c>
       <c r="I606">
         <v>9.09</v>
@@ -19924,7 +20578,7 @@
         <v>69.44</v>
       </c>
       <c r="I607">
-        <v>9.960000000000001</v>
+        <v>9.96</v>
       </c>
       <c r="J607">
         <v>20.6</v>
@@ -19953,7 +20607,7 @@
         <v>558.15</v>
       </c>
       <c r="H608">
-        <v>67.40000000000001</v>
+        <v>67.4</v>
       </c>
       <c r="I608">
         <v>10.43</v>
@@ -19985,7 +20639,7 @@
         <v>609.3</v>
       </c>
       <c r="H609">
-        <v>65.40000000000001</v>
+        <v>65.4</v>
       </c>
       <c r="I609">
         <v>10.9</v>
@@ -20552,7 +21206,7 @@
         <v>126.33</v>
       </c>
       <c r="E627">
-        <v>89.65000000000001</v>
+        <v>89.65</v>
       </c>
       <c r="F627">
         <v>8.16</v>
@@ -20587,7 +21241,7 @@
         <v>89.63</v>
       </c>
       <c r="F628">
-        <v>8.109999999999999</v>
+        <v>8.11</v>
       </c>
       <c r="G628">
         <v>32.46</v>
@@ -20625,10 +21279,10 @@
         <v>35.31</v>
       </c>
       <c r="H629">
-        <v>64.09999999999999</v>
+        <v>64.1</v>
       </c>
       <c r="I629">
-        <v>9.300000000000001</v>
+        <v>9.3</v>
       </c>
       <c r="J629">
         <v>26.6</v>
@@ -20712,7 +21366,7 @@
         <v>148.2</v>
       </c>
       <c r="E632">
-        <v>87.31999999999999</v>
+        <v>87.32</v>
       </c>
       <c r="F632">
         <v>14.28</v>
@@ -20936,13 +21590,13 @@
         <v>175.01</v>
       </c>
       <c r="E639">
-        <v>78.93000000000001</v>
+        <v>78.93</v>
       </c>
       <c r="F639">
         <v>24.68</v>
       </c>
       <c r="G639">
-        <v>71.40000000000001</v>
+        <v>71.4</v>
       </c>
       <c r="H639">
         <v>45.1</v>
@@ -21000,7 +21654,7 @@
         <v>181</v>
       </c>
       <c r="E641">
-        <v>74.56999999999999</v>
+        <v>74.57</v>
       </c>
       <c r="F641">
         <v>24.07</v>
@@ -21032,7 +21686,7 @@
         <v>185</v>
       </c>
       <c r="E642">
-        <v>69.79000000000001</v>
+        <v>69.79</v>
       </c>
       <c r="F642">
         <v>30.38</v>
@@ -21070,7 +21724,7 @@
         <v>33.1</v>
       </c>
       <c r="G643">
-        <v>84.15000000000001</v>
+        <v>84.15</v>
       </c>
       <c r="H643">
         <v>37.3</v>
@@ -21128,13 +21782,13 @@
         <v>190</v>
       </c>
       <c r="E645">
-        <v>67.73999999999999</v>
+        <v>67.74</v>
       </c>
       <c r="F645">
         <v>41.3</v>
       </c>
       <c r="G645">
-        <v>80.95999999999999</v>
+        <v>80.96</v>
       </c>
       <c r="H645">
         <v>35.7</v>
@@ -21658,7 +22312,7 @@
         <v>31.5764</v>
       </c>
     </row>
-    <row r="662" spans="1:10">
+    <row r="662" spans="1:7">
       <c r="A662" s="1">
         <v>1829</v>
       </c>
@@ -21713,7 +22367,7 @@
         <v>23.0622009569378</v>
       </c>
     </row>
-    <row r="664" spans="1:10">
+    <row r="664" spans="1:7">
       <c r="A664" s="1">
         <v>1831</v>
       </c>
@@ -21736,7 +22390,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="665" spans="1:10">
+    <row r="665" spans="1:7">
       <c r="A665" s="1">
         <v>1832</v>
       </c>
@@ -21759,7 +22413,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="666" spans="1:10">
+    <row r="666" spans="1:7">
       <c r="A666" s="1">
         <v>1833</v>
       </c>
@@ -21782,7 +22436,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="667" spans="1:10">
+    <row r="667" spans="1:7">
       <c r="A667" s="1">
         <v>1834</v>
       </c>
@@ -21805,7 +22459,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="668" spans="1:10">
+    <row r="668" spans="1:7">
       <c r="A668" s="1">
         <v>1835</v>
       </c>
@@ -21828,7 +22482,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="669" spans="1:10">
+    <row r="669" spans="1:7">
       <c r="A669" s="1">
         <v>1836</v>
       </c>
@@ -21993,7 +22647,7 @@
         <v>1476.45</v>
       </c>
       <c r="E674">
-        <v>880.5599999999999</v>
+        <v>880.56</v>
       </c>
       <c r="F674">
         <v>279.78</v>
@@ -22153,7 +22807,7 @@
         <v>1391.36</v>
       </c>
       <c r="E679">
-        <v>885.8200000000001</v>
+        <v>885.82</v>
       </c>
       <c r="F679">
         <v>203.96</v>
@@ -22313,7 +22967,7 @@
         <v>1397</v>
       </c>
       <c r="E684">
-        <v>860.6926999999999</v>
+        <v>860.6927</v>
       </c>
       <c r="F684">
         <v>214.5769</v>
@@ -22831,7 +23485,7 @@
         <v>39.13</v>
       </c>
       <c r="G700">
-        <v>86.31999999999999</v>
+        <v>86.32</v>
       </c>
       <c r="H700">
         <v>56.4</v>
@@ -23244,7 +23898,7 @@
         <v>115.09</v>
       </c>
       <c r="F713">
-        <v>73.93000000000001</v>
+        <v>73.93</v>
       </c>
       <c r="G713">
         <v>132.39</v>
@@ -23663,7 +24317,7 @@
         <v>63.5</v>
       </c>
       <c r="G726">
-        <v>85.90000000000001</v>
+        <v>85.9</v>
       </c>
       <c r="H726">
         <v>49.8</v>
@@ -23695,7 +24349,7 @@
         <v>66.73</v>
       </c>
       <c r="G727">
-        <v>87.79000000000001</v>
+        <v>87.79</v>
       </c>
       <c r="H727">
         <v>48.4</v>
@@ -23724,10 +24378,10 @@
         <v>140.1</v>
       </c>
       <c r="F728">
-        <v>72.09999999999999</v>
+        <v>72.1</v>
       </c>
       <c r="G728">
-        <v>95.90000000000001</v>
+        <v>95.9</v>
       </c>
       <c r="H728">
         <v>45.5</v>
@@ -23756,7 +24410,7 @@
         <v>141.5</v>
       </c>
       <c r="F729">
-        <v>70.09999999999999</v>
+        <v>70.1</v>
       </c>
       <c r="G729">
         <v>97.8</v>
@@ -23791,7 +24445,7 @@
         <v>76.2</v>
       </c>
       <c r="G730">
-        <v>91.40000000000001</v>
+        <v>91.4</v>
       </c>
       <c r="H730">
         <v>44.9</v>
@@ -24012,7 +24666,7 @@
         <v>125.5</v>
       </c>
       <c r="F737">
-        <v>80.59999999999999</v>
+        <v>80.6</v>
       </c>
       <c r="G737">
         <v>136.9</v>
@@ -24137,7 +24791,7 @@
         <v>343</v>
       </c>
       <c r="E741">
-        <v>90.59999999999999</v>
+        <v>90.6</v>
       </c>
       <c r="F741">
         <v>81.3</v>
@@ -24364,7 +25018,7 @@
         <v>391.84</v>
       </c>
       <c r="F748">
-        <v>95.81999999999999</v>
+        <v>95.82</v>
       </c>
       <c r="G748">
         <v>213.83</v>
@@ -24428,7 +25082,7 @@
         <v>403.31</v>
       </c>
       <c r="F750">
-        <v>98.48999999999999</v>
+        <v>98.49</v>
       </c>
       <c r="G750">
         <v>242.69</v>
@@ -24847,7 +25501,7 @@
         <v>192.65</v>
       </c>
       <c r="G763">
-        <v>584.4400000000001</v>
+        <v>584.44</v>
       </c>
       <c r="H763">
         <v>40.88</v>
@@ -25053,5 +25707,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>